<commit_message>
Dashboard: 2026-07-07 12:58 UTC
</commit_message>
<xml_diff>
--- a/instagram-metrics/base_interacoes_detalhadas.xlsx
+++ b/instagram-metrics/base_interacoes_detalhadas.xlsx
@@ -956,69 +956,69 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>06/07/2026</t>
+          <t>07/07/2026</t>
         </is>
       </c>
       <c r="E12" s="2" t="n">
-        <v>0</v>
+        <v>627</v>
       </c>
       <c r="F12" s="2" t="n">
-        <v>0</v>
+        <v>61</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>0</v>
+        <v>81</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>0</v>
+        <v>45</v>
       </c>
       <c r="I12" s="2" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06 20:32</t>
+          <t>2026-07-07 12:57</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="3" t="inlineStr">
+      <c r="A13" s="2" t="inlineStr">
         <is>
           <t>S28/2026</t>
         </is>
       </c>
-      <c r="B13" s="3" t="inlineStr">
+      <c r="B13" s="2" t="inlineStr">
         <is>
           <t>Personal</t>
         </is>
       </c>
-      <c r="C13" s="3" t="inlineStr">
-        <is>
-          <t>01/07/2026</t>
-        </is>
-      </c>
-      <c r="D13" s="3" t="inlineStr">
-        <is>
-          <t>06/07/2026</t>
-        </is>
-      </c>
-      <c r="E13" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="F13" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="G13" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H13" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="I13" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="J13" s="3" t="inlineStr">
-        <is>
-          <t>2026-07-06 20:32</t>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>01/07/2026</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>07/07/2026</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="n">
+        <v>64</v>
+      </c>
+      <c r="F13" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G13" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="H13" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="I13" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-07 12:57</t>
         </is>
       </c>
     </row>
@@ -1040,69 +1040,69 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>06/07/2026</t>
+          <t>07/07/2026</t>
         </is>
       </c>
       <c r="E14" s="2" t="n">
-        <v>0</v>
+        <v>203</v>
       </c>
       <c r="F14" s="2" t="n">
-        <v>0</v>
+        <v>52</v>
       </c>
       <c r="G14" s="2" t="n">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="H14" s="2" t="n">
         <v>0</v>
       </c>
       <c r="I14" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06 20:32</t>
+          <t>2026-07-07 12:57</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="3" t="inlineStr">
+      <c r="A15" s="2" t="inlineStr">
         <is>
           <t>S28/2026</t>
         </is>
       </c>
-      <c r="B15" s="3" t="inlineStr">
+      <c r="B15" s="2" t="inlineStr">
         <is>
           <t>Family</t>
         </is>
       </c>
-      <c r="C15" s="3" t="inlineStr">
-        <is>
-          <t>01/07/2026</t>
-        </is>
-      </c>
-      <c r="D15" s="3" t="inlineStr">
-        <is>
-          <t>06/07/2026</t>
-        </is>
-      </c>
-      <c r="E15" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="F15" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="G15" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H15" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="I15" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="J15" s="3" t="inlineStr">
-        <is>
-          <t>2026-07-06 20:32</t>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>01/07/2026</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>07/07/2026</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="n">
+        <v>115</v>
+      </c>
+      <c r="F15" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="G15" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="H15" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="I15" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-07 12:57</t>
         </is>
       </c>
     </row>
@@ -1124,27 +1124,27 @@
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>06/07/2026</t>
+          <t>07/07/2026</t>
         </is>
       </c>
       <c r="E16" s="2" t="n">
-        <v>0</v>
+        <v>372</v>
       </c>
       <c r="F16" s="2" t="n">
-        <v>0</v>
+        <v>38</v>
       </c>
       <c r="G16" s="2" t="n">
-        <v>0</v>
+        <v>52</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="I16" s="2" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06 20:32</t>
+          <t>2026-07-07 12:57</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix: remove S28 São Paulo para forçar recoleta com novo token
</commit_message>
<xml_diff>
--- a/instagram-metrics/base_interacoes_detalhadas.xlsx
+++ b/instagram-metrics/base_interacoes_detalhadas.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Dados" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dados" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -451,7 +451,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J16"/>
+  <dimension ref="A1:J15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1030,7 +1030,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>São Paulo</t>
+          <t>Family</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -1044,16 +1044,16 @@
         </is>
       </c>
       <c r="E14" s="2" t="n">
-        <v>203</v>
+        <v>115</v>
       </c>
       <c r="F14" s="2" t="n">
-        <v>52</v>
+        <v>12</v>
       </c>
       <c r="G14" s="2" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="I14" s="2" t="n">
         <v>3</v>
@@ -1072,7 +1072,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Family</t>
+          <t>CT</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -1086,63 +1086,21 @@
         </is>
       </c>
       <c r="E15" s="2" t="n">
-        <v>115</v>
+        <v>372</v>
       </c>
       <c r="F15" s="2" t="n">
-        <v>12</v>
+        <v>38</v>
       </c>
       <c r="G15" s="2" t="n">
-        <v>21</v>
+        <v>52</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="I15" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J15" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-07 12:57</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>S28/2026</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>CT</t>
-        </is>
-      </c>
-      <c r="C16" s="2" t="inlineStr">
-        <is>
-          <t>01/07/2026</t>
-        </is>
-      </c>
-      <c r="D16" s="2" t="inlineStr">
-        <is>
-          <t>07/07/2026</t>
-        </is>
-      </c>
-      <c r="E16" s="2" t="n">
-        <v>372</v>
-      </c>
-      <c r="F16" s="2" t="n">
-        <v>38</v>
-      </c>
-      <c r="G16" s="2" t="n">
-        <v>52</v>
-      </c>
-      <c r="H16" s="2" t="n">
-        <v>11</v>
-      </c>
-      <c r="I16" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="J16" s="2" t="inlineStr">
         <is>
           <t>2026-07-07 12:57</t>
         </is>

</xml_diff>

<commit_message>
Fix: remove S28 completo para forçar recoleta com token SP correto
</commit_message>
<xml_diff>
--- a/instagram-metrics/base_interacoes_detalhadas.xlsx
+++ b/instagram-metrics/base_interacoes_detalhadas.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Dados" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dados" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -451,7 +451,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J16"/>
+  <dimension ref="A1:J11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -938,216 +938,6 @@
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>S28/2026</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>Academias</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>01/07/2026</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>09/07/2026</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="n">
-        <v>747</v>
-      </c>
-      <c r="F12" s="2" t="n">
-        <v>82</v>
-      </c>
-      <c r="G12" s="2" t="n">
-        <v>104</v>
-      </c>
-      <c r="H12" s="2" t="n">
-        <v>107</v>
-      </c>
-      <c r="I12" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="J12" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-09 13:42</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>S28/2026</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>Personal</t>
-        </is>
-      </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>01/07/2026</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>09/07/2026</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="n">
-        <v>71</v>
-      </c>
-      <c r="F13" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="G13" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="H13" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="I13" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="J13" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-09 13:42</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>S28/2026</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>São Paulo</t>
-        </is>
-      </c>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
-          <t>01/07/2026</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="inlineStr">
-        <is>
-          <t>09/07/2026</t>
-        </is>
-      </c>
-      <c r="E14" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F14" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G14" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H14" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I14" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J14" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-09 13:42</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>S28/2026</t>
-        </is>
-      </c>
-      <c r="B15" s="2" t="inlineStr">
-        <is>
-          <t>Family</t>
-        </is>
-      </c>
-      <c r="C15" s="2" t="inlineStr">
-        <is>
-          <t>01/07/2026</t>
-        </is>
-      </c>
-      <c r="D15" s="2" t="inlineStr">
-        <is>
-          <t>09/07/2026</t>
-        </is>
-      </c>
-      <c r="E15" s="2" t="n">
-        <v>145</v>
-      </c>
-      <c r="F15" s="2" t="n">
-        <v>22</v>
-      </c>
-      <c r="G15" s="2" t="n">
-        <v>28</v>
-      </c>
-      <c r="H15" s="2" t="n">
-        <v>79</v>
-      </c>
-      <c r="I15" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="J15" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-09 13:42</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>S28/2026</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>CT</t>
-        </is>
-      </c>
-      <c r="C16" s="2" t="inlineStr">
-        <is>
-          <t>01/07/2026</t>
-        </is>
-      </c>
-      <c r="D16" s="2" t="inlineStr">
-        <is>
-          <t>09/07/2026</t>
-        </is>
-      </c>
-      <c r="E16" s="2" t="n">
-        <v>543</v>
-      </c>
-      <c r="F16" s="2" t="n">
-        <v>53</v>
-      </c>
-      <c r="G16" s="2" t="n">
-        <v>63</v>
-      </c>
-      <c r="H16" s="2" t="n">
-        <v>16</v>
-      </c>
-      <c r="I16" s="2" t="n">
-        <v>6</v>
-      </c>
-      <c r="J16" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-09 13:42</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>